<commit_message>
v2: Restructured into src architecture with services, core, config and utils folders
</commit_message>
<xml_diff>
--- a/leads.xlsx
+++ b/leads.xlsx
@@ -460,10 +460,10 @@
         <v>2024-01-01</v>
       </c>
       <c r="H2" t="str">
-        <v>CONSIDERING</v>
+        <v>INTERESTED</v>
       </c>
       <c r="I2" t="str">
-        <v>2026-09-24</v>
+        <v>2026-09-25</v>
       </c>
       <c r="J2">
         <v>0</v>
@@ -498,10 +498,10 @@
         <v>2024-01-01</v>
       </c>
       <c r="H3" t="str">
-        <v>CONSIDERING</v>
+        <v>INTERESTED</v>
       </c>
       <c r="I3" t="str">
-        <v>2026-09-24</v>
+        <v>2026-09-25</v>
       </c>
       <c r="J3">
         <v>0</v>
@@ -536,10 +536,10 @@
         <v>2024-01-01</v>
       </c>
       <c r="H4" t="str">
-        <v>CONSIDERING</v>
+        <v>INTERESTED</v>
       </c>
       <c r="I4" t="str">
-        <v>2026-09-24</v>
+        <v>2026-09-25</v>
       </c>
       <c r="J4">
         <v>0</v>

</xml_diff>